<commit_message>
Merging fueldata and storagedata to nodedata. Clarifying assumptions that in source excel pipeline NA is no data and zero mean data, but in input excel data pipeline empty = NA = zero.
</commit_message>
<xml_diff>
--- a/src_files/data_files/Finland_dheat_and_industry.xlsx
+++ b/src_files/data_files/Finland_dheat_and_industry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-master\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A0393F9-7D5A-4565-8D61-44C1C3BFD061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5C5503-A39A-4DAB-8E22-BD7EEEDD37C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="889" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="889" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="demanddata_FI-industry" sheetId="16" r:id="rId1"/>

</xml_diff>

<commit_message>
Removing <10 MW units, additing purchase power differentiated vomCosts to units, updating the layout of files, sorting rows.
</commit_message>
<xml_diff>
--- a/src_files/data_files/Finland_dheat_and_industry.xlsx
+++ b/src_files/data_files/Finland_dheat_and_industry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-master\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5C5503-A39A-4DAB-8E22-BD7EEEDD37C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BACF4D0-5709-4F1C-A58E-A2FE0815E2EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="889" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-18120" yWindow="-105" windowWidth="18240" windowHeight="28320" tabRatio="889" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="demanddata_FI-industry" sheetId="16" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9542" uniqueCount="1643">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9534" uniqueCount="1642">
   <si>
     <t>Country</t>
   </si>
@@ -4987,9 +4987,6 @@
   </si>
   <si>
     <t>method</t>
-  </si>
-  <si>
-    <t>remove</t>
   </si>
   <si>
     <t>variableTransCost</t>
@@ -5476,7 +5473,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -5727,6 +5724,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -51468,13 +51466,13 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="91" t="s">
-        <v>1641</v>
+        <v>1640</v>
       </c>
       <c r="B1" s="91" t="s">
         <v>1629</v>
       </c>
       <c r="C1" s="91" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="D1" s="91" t="s">
         <v>1630</v>
@@ -51489,16 +51487,16 @@
         <v>3</v>
       </c>
       <c r="H1" s="92" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="I1" s="92" t="s">
         <v>1633</v>
       </c>
       <c r="J1" s="92" t="s">
+        <v>1637</v>
+      </c>
+      <c r="K1" s="92" t="s">
         <v>1638</v>
-      </c>
-      <c r="K1" s="92" t="s">
-        <v>1639</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -52557,6 +52555,10 @@
         <f ca="1">IF(ISNUMBER($F2),($H2+$J2)/$F2,"")</f>
         <v/>
       </c>
+      <c r="Q2" s="98" t="str">
+        <f ca="1">IF(H2&lt;10, "remove", "")</f>
+        <v/>
+      </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" t="s">
@@ -52611,6 +52613,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q3" s="98" t="str">
+        <f t="shared" ref="Q3:Q66" ca="1" si="5">IF(H3&lt;10, "remove", "")</f>
+        <v/>
+      </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" t="s">
@@ -52665,6 +52671,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q4" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
@@ -52717,6 +52727,10 @@
       </c>
       <c r="O5" s="46" t="str">
         <f t="shared" ca="1" si="4"/>
+        <v/>
+      </c>
+      <c r="Q5" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
     </row>
@@ -52773,6 +52787,10 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.90618019359642588</v>
       </c>
+      <c r="Q6" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
@@ -52827,6 +52845,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q7" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
@@ -52881,6 +52903,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q8" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" t="s">
@@ -52935,6 +52961,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q9" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" t="s">
@@ -52989,6 +53019,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q10" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
@@ -53043,6 +53077,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q11" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" t="s">
@@ -53097,6 +53135,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q12" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" t="s">
@@ -53151,6 +53193,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q13" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" t="s">
@@ -53205,6 +53251,10 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
+      <c r="Q14" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" t="s">
@@ -53257,6 +53307,10 @@
       </c>
       <c r="O15" s="46" t="str">
         <f t="shared" ca="1" si="4"/>
+        <v/>
+      </c>
+      <c r="Q15" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
     </row>
@@ -53313,8 +53367,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.89759036144578308</v>
       </c>
-    </row>
-    <row r="17" spans="1:15">
+      <c r="Q16" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -53367,8 +53425,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.97727272727272729</v>
       </c>
-    </row>
-    <row r="18" spans="1:15">
+      <c r="Q17" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -53421,8 +53483,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="19" spans="1:15">
+      <c r="Q18" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -53475,8 +53541,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="20" spans="1:15">
+      <c r="Q19" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -53529,8 +53599,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="21" spans="1:15">
+      <c r="Q20" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -53583,8 +53657,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="22" spans="1:15">
+      <c r="Q21" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -53637,8 +53715,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="23" spans="1:15">
+      <c r="Q22" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -53691,8 +53773,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="24" spans="1:15">
+      <c r="Q23" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -53745,8 +53831,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.80909090909090908</v>
       </c>
-    </row>
-    <row r="25" spans="1:15">
+      <c r="Q24" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -53799,8 +53889,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>1.1083333333333334</v>
       </c>
-    </row>
-    <row r="26" spans="1:15">
+      <c r="Q25" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" t="s">
         <v>17</v>
       </c>
@@ -53853,8 +53947,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>1.105940594059406</v>
       </c>
-    </row>
-    <row r="27" spans="1:15">
+      <c r="Q26" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -53907,8 +54005,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="28" spans="1:15">
+      <c r="Q27" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" t="s">
         <v>17</v>
       </c>
@@ -53961,8 +54063,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="29" spans="1:15">
+      <c r="Q28" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" t="s">
         <v>17</v>
       </c>
@@ -54015,8 +54121,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="30" spans="1:15">
+      <c r="Q29" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -54069,8 +54179,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="31" spans="1:15">
+      <c r="Q30" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" t="s">
         <v>17</v>
       </c>
@@ -54123,8 +54237,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="32" spans="1:15">
+      <c r="Q31" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" t="s">
         <v>17</v>
       </c>
@@ -54177,8 +54295,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="33" spans="1:15">
+      <c r="Q32" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" t="s">
         <v>17</v>
       </c>
@@ -54231,8 +54353,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="34" spans="1:15">
+      <c r="Q33" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" t="s">
         <v>17</v>
       </c>
@@ -54285,8 +54411,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="35" spans="1:15">
+      <c r="Q34" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" t="s">
         <v>17</v>
       </c>
@@ -54339,8 +54469,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="36" spans="1:15">
+      <c r="Q35" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -54393,8 +54527,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="37" spans="1:15">
+      <c r="Q36" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" t="s">
         <v>17</v>
       </c>
@@ -54447,8 +54585,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="38" spans="1:15">
+      <c r="Q37" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" t="s">
         <v>17</v>
       </c>
@@ -54501,8 +54643,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>1.0238095238095237</v>
       </c>
-    </row>
-    <row r="39" spans="1:15">
+      <c r="Q38" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" t="s">
         <v>17</v>
       </c>
@@ -54555,8 +54701,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.94345238095238093</v>
       </c>
-    </row>
-    <row r="40" spans="1:15">
+      <c r="Q39" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" t="s">
         <v>17</v>
       </c>
@@ -54609,8 +54759,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.87878787878787878</v>
       </c>
-    </row>
-    <row r="41" spans="1:15">
+      <c r="Q40" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" t="s">
         <v>17</v>
       </c>
@@ -54663,8 +54817,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="42" spans="1:15">
+      <c r="Q41" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -54717,8 +54875,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="43" spans="1:15">
+      <c r="Q42" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" t="s">
         <v>17</v>
       </c>
@@ -54771,8 +54933,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="44" spans="1:15">
+      <c r="Q43" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" t="s">
         <v>17</v>
       </c>
@@ -54825,8 +54991,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="45" spans="1:15">
+      <c r="Q44" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" t="s">
         <v>17</v>
       </c>
@@ -54879,8 +55049,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="46" spans="1:15">
+      <c r="Q45" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v>remove</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" t="s">
         <v>17</v>
       </c>
@@ -54933,8 +55107,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>1.0320754716981133</v>
       </c>
-    </row>
-    <row r="47" spans="1:15">
+      <c r="Q46" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" t="s">
         <v>17</v>
       </c>
@@ -54987,8 +55165,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="48" spans="1:15">
+      <c r="Q47" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" t="s">
         <v>17</v>
       </c>
@@ -55041,8 +55223,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="49" spans="1:15">
+      <c r="Q48" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" t="s">
         <v>17</v>
       </c>
@@ -55095,8 +55281,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="50" spans="1:15">
+      <c r="Q49" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" t="s">
         <v>17</v>
       </c>
@@ -55149,8 +55339,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="51" spans="1:15">
+      <c r="Q50" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" t="s">
         <v>17</v>
       </c>
@@ -55203,8 +55397,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="52" spans="1:15">
+      <c r="Q51" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" t="s">
         <v>17</v>
       </c>
@@ -55257,8 +55455,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="53" spans="1:15">
+      <c r="Q52" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" t="s">
         <v>17</v>
       </c>
@@ -55311,8 +55513,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="54" spans="1:15">
+      <c r="Q53" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" t="s">
         <v>17</v>
       </c>
@@ -55365,8 +55571,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.99056603773584906</v>
       </c>
-    </row>
-    <row r="55" spans="1:15">
+      <c r="Q54" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" t="s">
         <v>17</v>
       </c>
@@ -55419,8 +55629,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="56" spans="1:15">
+      <c r="Q55" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" t="s">
         <v>17</v>
       </c>
@@ -55473,8 +55687,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="57" spans="1:15">
+      <c r="Q56" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" t="s">
         <v>17</v>
       </c>
@@ -55527,8 +55745,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="58" spans="1:15">
+      <c r="Q57" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" t="s">
         <v>17</v>
       </c>
@@ -55581,8 +55803,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="59" spans="1:15">
+      <c r="Q58" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" t="s">
         <v>17</v>
       </c>
@@ -55635,8 +55861,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="60" spans="1:15">
+      <c r="Q59" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v>remove</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60" t="s">
         <v>17</v>
       </c>
@@ -55689,8 +55919,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="61" spans="1:15">
+      <c r="Q60" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61" t="s">
         <v>17</v>
       </c>
@@ -55743,8 +55977,12 @@
         <f t="shared" ca="1" si="4"/>
         <v>0.86708860759493667</v>
       </c>
-    </row>
-    <row r="62" spans="1:15">
+      <c r="Q61" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" t="s">
         <v>17</v>
       </c>
@@ -55797,8 +56035,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="63" spans="1:15">
+      <c r="Q62" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -55851,8 +56093,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="64" spans="1:15">
+      <c r="Q63" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" t="s">
         <v>17</v>
       </c>
@@ -55905,8 +56151,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="65" spans="1:15">
+      <c r="Q64" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" t="s">
         <v>17</v>
       </c>
@@ -55959,8 +56209,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="66" spans="1:15">
+      <c r="Q65" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" t="s">
         <v>17</v>
       </c>
@@ -56001,7 +56255,7 @@
         <v/>
       </c>
       <c r="L66" s="46" t="str">
-        <f t="shared" ref="L66:L81" ca="1" si="5">IF(ISTEXT($B66),IF($J66&gt;0,$H66/$J66,""),"")</f>
+        <f t="shared" ref="L66:L81" ca="1" si="6">IF(ISTEXT($B66),IF($J66&gt;0,$H66/$J66,""),"")</f>
         <v/>
       </c>
       <c r="M66" s="46"/>
@@ -56013,8 +56267,12 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-    </row>
-    <row r="67" spans="1:15">
+      <c r="Q66" s="98" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" t="s">
         <v>17</v>
       </c>
@@ -56035,7 +56293,7 @@
         <v/>
       </c>
       <c r="G67" s="46" t="str">
-        <f t="shared" ref="G67:G81" si="6">IF(COUNTIF($B67,"*charger*"),$C67,"")</f>
+        <f t="shared" ref="G67:G81" si="7">IF(COUNTIF($B67,"*charger*"),$C67,"")</f>
         <v/>
       </c>
       <c r="H67" s="46">
@@ -56043,7 +56301,7 @@
         <v>10</v>
       </c>
       <c r="I67" s="46" t="str">
-        <f t="shared" ref="I67:I81" si="7">IF(COUNTIF($B67,"*HOB*")+COUNTIF($B67,"*charger*")+COUNTIF($B67,"*heat pump*")+COUNTIF($B67,"electric boiler"),C67,"")</f>
+        <f t="shared" ref="I67:I81" si="8">IF(COUNTIF($B67,"*HOB*")+COUNTIF($B67,"*charger*")+COUNTIF($B67,"*heat pump*")+COUNTIF($B67,"electric boiler"),C67,"")</f>
         <v>ROF</v>
       </c>
       <c r="J67" s="46">
@@ -56051,24 +56309,28 @@
         <v>0</v>
       </c>
       <c r="K67" s="46" t="str">
-        <f t="shared" ref="K67:K81" ca="1" si="8">IF(J67=0,"",IF(ISTEXT($B67),IF(COUNTIF($B67,"*Industry*"),"industry",$C67),""))</f>
+        <f t="shared" ref="K67:K81" ca="1" si="9">IF(J67=0,"",IF(ISTEXT($B67),IF(COUNTIF($B67,"*Industry*"),"industry",$C67),""))</f>
         <v/>
       </c>
       <c r="L67" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M67" s="46"/>
       <c r="N67" s="46" t="str">
-        <f t="shared" ref="N67:O81" ca="1" si="9">IF(ISNUMBER($F67),($H67+$J67)/$F67,"")</f>
+        <f t="shared" ref="N67:O81" ca="1" si="10">IF(ISNUMBER($F67),($H67+$J67)/$F67,"")</f>
         <v/>
       </c>
       <c r="O67" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q67" s="98" t="str">
+        <f t="shared" ref="Q67:Q89" ca="1" si="11">IF(H67&lt;10, "remove", "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" t="s">
         <v>17</v>
       </c>
@@ -56089,7 +56351,7 @@
         <v/>
       </c>
       <c r="G68" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H68" s="46">
@@ -56097,7 +56359,7 @@
         <v>2701.9000000000005</v>
       </c>
       <c r="I68" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J68" s="46">
@@ -56105,24 +56367,28 @@
         <v>0</v>
       </c>
       <c r="K68" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L68" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M68" s="46"/>
       <c r="N68" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O68" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q68" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" t="s">
         <v>17</v>
       </c>
@@ -56143,7 +56409,7 @@
         <v/>
       </c>
       <c r="G69" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H69" s="46">
@@ -56151,7 +56417,7 @@
         <v>1426.6</v>
       </c>
       <c r="I69" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J69" s="46">
@@ -56159,24 +56425,28 @@
         <v>3099.2999999999997</v>
       </c>
       <c r="K69" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v>ROF</v>
       </c>
       <c r="L69" s="46">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v>0.46029748652921626</v>
       </c>
       <c r="M69" s="46"/>
       <c r="N69" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O69" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q69" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" t="s">
         <v>17</v>
       </c>
@@ -56197,7 +56467,7 @@
         <v/>
       </c>
       <c r="G70" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H70" s="46">
@@ -56205,7 +56475,7 @@
         <v>1849.9999999999998</v>
       </c>
       <c r="I70" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J70" s="46">
@@ -56213,24 +56483,28 @@
         <v>0</v>
       </c>
       <c r="K70" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L70" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M70" s="46"/>
       <c r="N70" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O70" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q70" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" t="s">
         <v>17</v>
       </c>
@@ -56251,7 +56525,7 @@
         <v/>
       </c>
       <c r="G71" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H71" s="46">
@@ -56259,7 +56533,7 @@
         <v>148.80000000000001</v>
       </c>
       <c r="I71" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J71" s="46">
@@ -56267,24 +56541,28 @@
         <v>0</v>
       </c>
       <c r="K71" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L71" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M71" s="46"/>
       <c r="N71" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O71" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q71" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" t="s">
         <v>17</v>
       </c>
@@ -56305,7 +56583,7 @@
         <v/>
       </c>
       <c r="G72" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H72" s="46">
@@ -56313,7 +56591,7 @@
         <v>211.3</v>
       </c>
       <c r="I72" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J72" s="46">
@@ -56321,24 +56599,28 @@
         <v>356.6</v>
       </c>
       <c r="K72" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v>ROF</v>
       </c>
       <c r="L72" s="46">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v>0.592540661805945</v>
       </c>
       <c r="M72" s="46"/>
       <c r="N72" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O72" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q72" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" t="s">
         <v>17</v>
       </c>
@@ -56359,7 +56641,7 @@
         <v/>
       </c>
       <c r="G73" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H73" s="46">
@@ -56367,7 +56649,7 @@
         <v>113.2</v>
       </c>
       <c r="I73" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J73" s="46">
@@ -56375,24 +56657,28 @@
         <v>345</v>
       </c>
       <c r="K73" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v>ROF</v>
       </c>
       <c r="L73" s="46">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v>0.32811594202898553</v>
       </c>
       <c r="M73" s="46"/>
       <c r="N73" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O73" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q73" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" t="s">
         <v>17</v>
       </c>
@@ -56413,7 +56699,7 @@
         <v/>
       </c>
       <c r="G74" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H74" s="46">
@@ -56421,7 +56707,7 @@
         <v>1042.8999999999999</v>
       </c>
       <c r="I74" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J74" s="46">
@@ -56429,24 +56715,28 @@
         <v>0</v>
       </c>
       <c r="K74" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L74" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M74" s="46"/>
       <c r="N74" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O74" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q74" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" t="s">
         <v>17</v>
       </c>
@@ -56467,7 +56757,7 @@
         <v/>
       </c>
       <c r="G75" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>ROF</v>
       </c>
       <c r="H75" s="46">
@@ -56475,7 +56765,7 @@
         <v>625.5</v>
       </c>
       <c r="I75" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J75" s="46">
@@ -56483,24 +56773,28 @@
         <v>0</v>
       </c>
       <c r="K75" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L75" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M75" s="46"/>
       <c r="N75" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O75" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q75" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" t="s">
         <v>17</v>
       </c>
@@ -56521,7 +56815,7 @@
         <v/>
       </c>
       <c r="G76" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>ROF</v>
       </c>
       <c r="H76" s="46">
@@ -56529,7 +56823,7 @@
         <v>625.5</v>
       </c>
       <c r="I76" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J76" s="46">
@@ -56537,24 +56831,28 @@
         <v>0</v>
       </c>
       <c r="K76" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L76" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M76" s="46"/>
       <c r="N76" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O76" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q76" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" t="s">
         <v>17</v>
       </c>
@@ -56575,7 +56873,7 @@
         <v/>
       </c>
       <c r="G77" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>ROF</v>
       </c>
       <c r="H77" s="46">
@@ -56583,7 +56881,7 @@
         <v>170</v>
       </c>
       <c r="I77" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J77" s="46">
@@ -56591,24 +56889,28 @@
         <v>0</v>
       </c>
       <c r="K77" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L77" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M77" s="46"/>
       <c r="N77" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O77" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q77" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" t="s">
         <v>17</v>
       </c>
@@ -56629,7 +56931,7 @@
         <v/>
       </c>
       <c r="G78" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>ROF</v>
       </c>
       <c r="H78" s="46">
@@ -56637,7 +56939,7 @@
         <v>170</v>
       </c>
       <c r="I78" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>ROF</v>
       </c>
       <c r="J78" s="46">
@@ -56645,24 +56947,28 @@
         <v>0</v>
       </c>
       <c r="K78" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="L78" s="46" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v/>
       </c>
       <c r="M78" s="46"/>
       <c r="N78" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v/>
       </c>
       <c r="O78" s="46" t="str">
-        <f t="shared" ca="1" si="9"/>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="1:15">
+        <f t="shared" ca="1" si="10"/>
+        <v/>
+      </c>
+      <c r="Q78" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" t="s">
         <v>17</v>
       </c>
@@ -56680,7 +56986,7 @@
         <v>8433.6666666666679</v>
       </c>
       <c r="G79" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H79" s="46">
@@ -56688,7 +56994,7 @@
         <v>2530.1000000000004</v>
       </c>
       <c r="I79" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J79" s="46">
@@ -56696,26 +57002,30 @@
         <v>5060.2000000000007</v>
       </c>
       <c r="K79" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v>industry</v>
       </c>
       <c r="L79" s="46">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v>0.5</v>
       </c>
       <c r="M79" s="46">
         <v>0</v>
       </c>
       <c r="N79" s="46">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0.9</v>
       </c>
       <c r="O79" s="46">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0.9</v>
       </c>
-    </row>
-    <row r="80" spans="1:15">
+      <c r="Q79" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" t="s">
         <v>17</v>
       </c>
@@ -56733,7 +57043,7 @@
         <v>650</v>
       </c>
       <c r="G80" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H80" s="46">
@@ -56741,7 +57051,7 @@
         <v>195</v>
       </c>
       <c r="I80" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J80" s="46">
@@ -56749,23 +57059,27 @@
         <v>390</v>
       </c>
       <c r="K80" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v>industry</v>
       </c>
       <c r="L80" s="46">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v>0.5</v>
       </c>
       <c r="M80" s="46">
         <v>0</v>
       </c>
       <c r="N80" s="46">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0.9</v>
       </c>
       <c r="O80" s="46">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0.9</v>
+      </c>
+      <c r="Q80" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
       </c>
     </row>
     <row r="81" spans="1:17">
@@ -56786,7 +57100,7 @@
         <v>1336.6666666666667</v>
       </c>
       <c r="G81" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H81" s="46">
@@ -56794,7 +57108,7 @@
         <v>401</v>
       </c>
       <c r="I81" s="46" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="J81" s="46">
@@ -56802,23 +57116,27 @@
         <v>802</v>
       </c>
       <c r="K81" s="46" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v>industry</v>
       </c>
       <c r="L81" s="46">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="6"/>
         <v>0.5</v>
       </c>
       <c r="M81" s="46">
         <v>0</v>
       </c>
       <c r="N81" s="46">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="O81" s="46">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="10"/>
         <v>0.89999999999999991</v>
+      </c>
+      <c r="Q81" s="98" t="str">
+        <f t="shared" ca="1" si="11"/>
+        <v/>
       </c>
     </row>
     <row r="82" spans="1:17">
@@ -56834,8 +57152,9 @@
       <c r="E82" s="53">
         <v>1</v>
       </c>
-      <c r="Q82" t="s">
-        <v>1637</v>
+      <c r="Q82" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="83" spans="1:17">
@@ -56851,8 +57170,9 @@
       <c r="E83" s="53">
         <v>1</v>
       </c>
-      <c r="Q83" t="s">
-        <v>1637</v>
+      <c r="Q83" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="84" spans="1:17">
@@ -56868,8 +57188,9 @@
       <c r="E84" s="53">
         <v>1</v>
       </c>
-      <c r="Q84" t="s">
-        <v>1637</v>
+      <c r="Q84" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="85" spans="1:17">
@@ -56885,8 +57206,9 @@
       <c r="E85" s="53">
         <v>1</v>
       </c>
-      <c r="Q85" t="s">
-        <v>1637</v>
+      <c r="Q85" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="86" spans="1:17">
@@ -56902,8 +57224,9 @@
       <c r="E86" s="53">
         <v>1</v>
       </c>
-      <c r="Q86" t="s">
-        <v>1637</v>
+      <c r="Q86" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="87" spans="1:17">
@@ -56919,8 +57242,9 @@
       <c r="E87" s="53">
         <v>1</v>
       </c>
-      <c r="Q87" t="s">
-        <v>1637</v>
+      <c r="Q87" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="88" spans="1:17">
@@ -56936,8 +57260,9 @@
       <c r="E88" s="53">
         <v>1</v>
       </c>
-      <c r="Q88" t="s">
-        <v>1637</v>
+      <c r="Q88" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
     <row r="89" spans="1:17">
@@ -56953,8 +57278,9 @@
       <c r="E89" s="53">
         <v>1</v>
       </c>
-      <c r="Q89" t="s">
-        <v>1637</v>
+      <c r="Q89" s="98" t="str">
+        <f t="shared" si="11"/>
+        <v>remove</v>
       </c>
     </row>
   </sheetData>

</xml_diff>